<commit_message>
fix: harden subcategory spreadsheet verification
</commit_message>
<xml_diff>
--- a/05_交付物/通俗细分版_2026-08-07/01_学术写作引用与出版/01-01_论文整体规划与流程管理/01-01_论文整体规划与流程管理_GitHub技能调研.xlsx
+++ b/05_交付物/通俗细分版_2026-08-07/01_学术写作引用与出版/01-01_论文整体规划与流程管理/01-01_论文整体规划与流程管理_GitHub技能调研.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="使用说明" sheetId="1" r:id="rId4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AI技能清单" sheetId="2" r:id="rId5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="分类统计" sheetId="3" r:id="rId6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="来源清单" sheetId="4" r:id="rId7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="使用说明" sheetId="1" r:id="R74ac0c09b08e41b5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AI技能清单" sheetId="2" r:id="Refbb3a19c4cd4227"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="分类统计" sheetId="3" r:id="Rf2799835c6334000"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="来源清单" sheetId="4" r:id="Rfb9b17f203644752"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1080,13 +1080,13 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:hyperlinks>
-    <x:hyperlink ref="U5" r:id="rId1"/>
-    <x:hyperlink ref="V5" r:id="rId2"/>
-    <x:hyperlink ref="U6" r:id="rId3"/>
-    <x:hyperlink ref="V6" r:id="rId4"/>
+    <x:hyperlink ref="U5" r:id="rIdHyperlink1"/>
+    <x:hyperlink ref="V5" r:id="rIdHyperlink2"/>
+    <x:hyperlink ref="U6" r:id="rIdHyperlink3"/>
+    <x:hyperlink ref="V6" r:id="rIdHyperlink4"/>
   </x:hyperlinks>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId5"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd0cc3612e787437e"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1358,11 +1358,11 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:hyperlinks>
-    <x:hyperlink ref="B5" r:id="rId1"/>
-    <x:hyperlink ref="B6" r:id="rId2"/>
+    <x:hyperlink ref="B5" r:id="rIdHyperlink1"/>
+    <x:hyperlink ref="B6" r:id="rIdHyperlink2"/>
   </x:hyperlinks>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId3"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc458a2308fc04fba"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
feat: generate complete subcategorized delivery
</commit_message>
<xml_diff>
--- a/05_交付物/通俗细分版_2026-08-07/01_学术写作引用与出版/01-01_论文整体规划与流程管理/01-01_论文整体规划与流程管理_GitHub技能调研.xlsx
+++ b/05_交付物/通俗细分版_2026-08-07/01_学术写作引用与出版/01-01_论文整体规划与流程管理/01-01_论文整体规划与流程管理_GitHub技能调研.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="使用说明" sheetId="1" r:id="R74ac0c09b08e41b5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AI技能清单" sheetId="2" r:id="Refbb3a19c4cd4227"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="分类统计" sheetId="3" r:id="Rf2799835c6334000"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="来源清单" sheetId="4" r:id="Rfb9b17f203644752"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="使用说明" sheetId="1" r:id="R1aeabc450be74001"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AI技能清单" sheetId="2" r:id="Rc640f612e9b148b2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="分类统计" sheetId="3" r:id="R6bac825c29924a3d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="来源清单" sheetId="4" r:id="Rf4119d1db3e346e6"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1086,7 +1086,7 @@
     <x:hyperlink ref="V6" r:id="rIdHyperlink4"/>
   </x:hyperlinks>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd0cc3612e787437e"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd1cfa9a9b7794140"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1362,7 +1362,7 @@
     <x:hyperlink ref="B6" r:id="rIdHyperlink2"/>
   </x:hyperlinks>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc458a2308fc04fba"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6939a4e6e84c4fdb"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>